<commit_message>
Change scoring column format in import assessment question xlsx file (#4915)
</commit_message>
<xml_diff>
--- a/public/example_csv/import_assessment_questions_sample_file.xlsx
+++ b/public/example_csv/import_assessment_questions_sample_file.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10114"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10811"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rohanpujari/tte/psychometrics/public/example_csv/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rohan-pujari/tte/psychometrics/public/example_csv/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0EE4022-D93D-E14D-9283-A68C9AEF6101}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C332960F-B080-1D41-AF6C-F70FEF5517DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2520" yWindow="1740" windowWidth="35120" windowHeight="22500" xr2:uid="{076B2D0F-1935-5E46-9497-2286E1A2EE28}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="67">
   <si>
     <t>Q1</t>
   </si>
@@ -98,9 +98,6 @@
     <t>answersType</t>
   </si>
   <si>
-    <t>Grit</t>
-  </si>
-  <si>
     <t>Yes</t>
   </si>
   <si>
@@ -143,9 +140,6 @@
     <t>Demonstrates agility to comfortably navigate uncertain and ambiguous situations.</t>
   </si>
   <si>
-    <t>1,2,1,2,1,2</t>
-  </si>
-  <si>
     <t>Q2</t>
   </si>
   <si>
@@ -212,9 +206,6 @@
     <t>EssayTextBox</t>
   </si>
   <si>
-    <t>Accountability</t>
-  </si>
-  <si>
     <t>Maybe</t>
   </si>
   <si>
@@ -227,31 +218,29 @@
     <t>All</t>
   </si>
   <si>
-    <t>3,2,4,6,3,5</t>
-  </si>
-  <si>
-    <t>1,3,2,2,4,2</t>
-  </si>
-  <si>
-    <t>1,2,4,4,3,5</t>
-  </si>
-  <si>
-    <t>1,2, 3</t>
-  </si>
-  <si>
-    <t>2, 4,5</t>
-  </si>
-  <si>
-    <t>3,2,1</t>
-  </si>
-  <si>
-    <t>4,5,6</t>
-  </si>
-  <si>
     <t>Static text Here</t>
   </si>
   <si>
     <t>PageBreak</t>
+  </si>
+  <si>
+    <t>Accountability: 1,2, 3
+Grit: 2, 4,5</t>
+  </si>
+  <si>
+    <t>Accountability: 3,2,1
+Grit: 4,5,6</t>
+  </si>
+  <si>
+    <t>Accountability: 1,2,1,2,1,2
+Grit: 3,2,4,6,3,5</t>
+  </si>
+  <si>
+    <t>Accountability: 1,3,2,2,4,2
+Grit: 1,2,4,4,3,5</t>
+  </si>
+  <si>
+    <t>Factors</t>
   </si>
 </sst>
 </file>
@@ -300,9 +289,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -637,7 +632,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2760F84-0E72-1247-B859-B08C7CC9D341}">
-  <dimension ref="A1:Q12"/>
+  <dimension ref="A1:P12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="16.83203125" customWidth="1"/>
@@ -655,7 +650,7 @@
     <col min="17" max="17" width="25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>10</v>
       </c>
@@ -699,16 +694,13 @@
         <v>12</v>
       </c>
       <c r="O1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="P1" t="s">
         <v>13</v>
       </c>
-      <c r="Q1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.2">
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -737,31 +729,28 @@
         <v>14</v>
       </c>
       <c r="J2" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="K2" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="L2" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="M2" t="s">
         <v>15</v>
       </c>
       <c r="N2" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="O2" t="s">
         <v>1</v>
       </c>
       <c r="P2" t="s">
-        <v>58</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.2">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -769,193 +758,187 @@
         <v>0</v>
       </c>
       <c r="C3" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D3" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="E3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="O3" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.2">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>16</v>
       </c>
       <c r="B4" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C4" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D4" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="O4" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.2">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>16</v>
       </c>
       <c r="B5" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C5" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E5" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.2">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" ht="34" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>17</v>
       </c>
       <c r="B6" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D6" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E6" t="s">
+        <v>24</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="H6" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="E6" t="s">
-        <v>25</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>44</v>
-      </c>
       <c r="I6" s="1" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="K6" s="1"/>
       <c r="L6" s="1"/>
       <c r="M6" t="s">
-        <v>44</v>
-      </c>
-      <c r="P6" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="Q6" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.2">
+        <v>42</v>
+      </c>
+      <c r="P6" s="2" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" ht="34" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>17</v>
       </c>
       <c r="B7" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="E7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="G7" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="H7" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="H7" s="1" t="s">
-        <v>23</v>
-      </c>
       <c r="I7" s="1" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="M7" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="N7">
         <v>1</v>
       </c>
-      <c r="P7" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="Q7" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="P7" s="2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>18</v>
       </c>
       <c r="B8" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>2</v>
       </c>
       <c r="E8" t="s">
+        <v>28</v>
+      </c>
+      <c r="G8" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="G8" s="1" t="s">
+      <c r="H8" s="1" t="s">
         <v>30</v>
-      </c>
-      <c r="H8" s="1" t="s">
-        <v>31</v>
       </c>
       <c r="I8" s="1"/>
       <c r="M8" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.2">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>18</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="D9" s="1"/>
       <c r="G9" s="1"/>
       <c r="H9" s="1"/>
       <c r="I9" s="1"/>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:16" ht="34" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>18</v>
       </c>
       <c r="B10" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>3</v>
       </c>
       <c r="E10" t="s">
+        <v>31</v>
+      </c>
+      <c r="F10" t="s">
+        <v>40</v>
+      </c>
+      <c r="G10" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="F10" t="s">
-        <v>42</v>
-      </c>
-      <c r="G10" s="1" t="s">
+      <c r="H10" s="1" t="s">
         <v>33</v>
-      </c>
-      <c r="H10" s="1" t="s">
-        <v>34</v>
       </c>
       <c r="I10" s="1"/>
       <c r="J10" s="1" t="s">
@@ -967,37 +950,34 @@
       <c r="L10" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="P10" t="s">
-        <v>35</v>
-      </c>
-      <c r="Q10" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="P10" s="3" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" ht="34" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>18</v>
       </c>
       <c r="B11" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D11" s="1" t="s">
         <v>3</v>
       </c>
       <c r="E11" t="s">
+        <v>31</v>
+      </c>
+      <c r="F11" t="s">
+        <v>41</v>
+      </c>
+      <c r="G11" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="F11" t="s">
-        <v>43</v>
-      </c>
-      <c r="G11" s="1" t="s">
+      <c r="H11" s="1" t="s">
         <v>33</v>
-      </c>
-      <c r="H11" s="1" t="s">
-        <v>34</v>
       </c>
       <c r="I11" s="1"/>
       <c r="J11" s="1" t="s">
@@ -1009,28 +989,25 @@
       <c r="L11" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="P11" t="s">
-        <v>64</v>
-      </c>
-      <c r="Q11" t="s">
+      <c r="P11" s="3" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>18</v>
       </c>
       <c r="B12" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="E12" t="s">
-        <v>70</v>
+        <v>60</v>
       </c>
       <c r="G12" s="1"/>
       <c r="H12" s="1"/>

</xml_diff>

<commit_message>
Add question import example file with all optipons (#5025)
</commit_message>
<xml_diff>
--- a/public/example_csv/import_assessment_questions_sample_file.xlsx
+++ b/public/example_csv/import_assessment_questions_sample_file.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rohan-pujari/tte/psychometrics/public/example_csv/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C332960F-B080-1D41-AF6C-F70FEF5517DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DB27CF3-E814-8443-B698-80752695E338}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2520" yWindow="1740" windowWidth="35120" windowHeight="22500" xr2:uid="{076B2D0F-1935-5E46-9497-2286E1A2EE28}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="33620" windowHeight="21580" xr2:uid="{076B2D0F-1935-5E46-9497-2286E1A2EE28}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="75">
   <si>
     <t>Q1</t>
   </si>
@@ -134,12 +134,6 @@
     <t>Demonstrating Strategic Vision</t>
   </si>
   <si>
-    <t>Translates organizational goals into meaningful actions to drive commitment to the company's strategy.</t>
-  </si>
-  <si>
-    <t>Demonstrates agility to comfortably navigate uncertain and ambiguous situations.</t>
-  </si>
-  <si>
     <t>Q2</t>
   </si>
   <si>
@@ -176,71 +170,99 @@
     <t>Force</t>
   </si>
   <si>
+    <t>Required Validation</t>
+  </si>
+  <si>
+    <t>Q8</t>
+  </si>
+  <si>
+    <t>StaticContent</t>
+  </si>
+  <si>
+    <t>TextEntry</t>
+  </si>
+  <si>
+    <t>MultipleChoice</t>
+  </si>
+  <si>
+    <t>MatrixTable</t>
+  </si>
+  <si>
+    <t>SingleLine</t>
+  </si>
+  <si>
+    <t>MultiLine</t>
+  </si>
+  <si>
+    <t>EssayTextBox</t>
+  </si>
+  <si>
+    <t>Maybe</t>
+  </si>
+  <si>
+    <t>Ireland</t>
+  </si>
+  <si>
+    <t>scalePointsTexts</t>
+  </si>
+  <si>
+    <t>All</t>
+  </si>
+  <si>
+    <t>Static text Here</t>
+  </si>
+  <si>
+    <t>PageBreak</t>
+  </si>
+  <si>
+    <t>Some</t>
+  </si>
+  <si>
     <t>Request</t>
   </si>
   <si>
-    <t>Required Validation</t>
-  </si>
-  <si>
-    <t>Q8</t>
-  </si>
-  <si>
-    <t>StaticContent</t>
-  </si>
-  <si>
-    <t>TextEntry</t>
-  </si>
-  <si>
-    <t>MultipleChoice</t>
-  </si>
-  <si>
-    <t>MatrixTable</t>
-  </si>
-  <si>
-    <t>SingleLine</t>
-  </si>
-  <si>
-    <t>MultiLine</t>
-  </si>
-  <si>
-    <t>EssayTextBox</t>
-  </si>
-  <si>
-    <t>Maybe</t>
-  </si>
-  <si>
-    <t>Ireland</t>
-  </si>
-  <si>
-    <t>scalePointsTexts</t>
-  </si>
-  <si>
-    <t>All</t>
-  </si>
-  <si>
-    <t>Static text Here</t>
-  </si>
-  <si>
-    <t>PageBreak</t>
-  </si>
-  <si>
-    <t>Accountability: 1,2, 3
+    <t>Q9</t>
+  </si>
+  <si>
+    <t>Agility</t>
+  </si>
+  <si>
+    <t>Commitment</t>
+  </si>
+  <si>
+    <t>Resilience</t>
+  </si>
+  <si>
+    <t>Disagree</t>
+  </si>
+  <si>
+    <t>Agree</t>
+  </si>
+  <si>
+    <t>Strongly Agree</t>
+  </si>
+  <si>
+    <t>Factors</t>
+  </si>
+  <si>
+    <t>notApplicable</t>
+  </si>
+  <si>
+    <t>notApplicableLabel</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>Q10</t>
+  </si>
+  <si>
+    <t>Accountability: 1,2,1,2,1,2
+Grit: ,,,4,,5</t>
+  </si>
+  <si>
+    <t>Accountability:1,, 3
 Grit: 2, 4,5</t>
-  </si>
-  <si>
-    <t>Accountability: 3,2,1
-Grit: 4,5,6</t>
-  </si>
-  <si>
-    <t>Accountability: 1,2,1,2,1,2
-Grit: 3,2,4,6,3,5</t>
-  </si>
-  <si>
-    <t>Accountability: 1,3,2,2,4,2
-Grit: 1,2,4,4,3,5</t>
-  </si>
-  <si>
-    <t>Factors</t>
   </si>
 </sst>
 </file>
@@ -632,7 +654,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2760F84-0E72-1247-B859-B08C7CC9D341}">
-  <dimension ref="A1:P12"/>
+  <dimension ref="A1:R13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="16.83203125" customWidth="1"/>
@@ -644,13 +666,13 @@
     <col min="8" max="9" width="27.33203125" customWidth="1"/>
     <col min="10" max="10" width="30.33203125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="21" customWidth="1"/>
-    <col min="12" max="12" width="25.83203125" customWidth="1"/>
-    <col min="13" max="15" width="37" customWidth="1"/>
-    <col min="16" max="16" width="24" customWidth="1"/>
-    <col min="17" max="17" width="25" bestFit="1" customWidth="1"/>
+    <col min="12" max="14" width="25.83203125" customWidth="1"/>
+    <col min="15" max="17" width="37" customWidth="1"/>
+    <col min="18" max="18" width="24" customWidth="1"/>
+    <col min="19" max="19" width="25" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>10</v>
       </c>
@@ -694,13 +716,19 @@
         <v>12</v>
       </c>
       <c r="O1" t="s">
-        <v>47</v>
+        <v>12</v>
       </c>
       <c r="P1" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>44</v>
+      </c>
+      <c r="R1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -729,28 +757,34 @@
         <v>14</v>
       </c>
       <c r="J2" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="K2" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="L2" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="M2" t="s">
+        <v>69</v>
+      </c>
+      <c r="N2" t="s">
+        <v>70</v>
+      </c>
+      <c r="O2" t="s">
         <v>15</v>
       </c>
-      <c r="N2" t="s">
-        <v>44</v>
-      </c>
-      <c r="O2" t="s">
+      <c r="P2" t="s">
+        <v>42</v>
+      </c>
+      <c r="Q2" t="s">
         <v>1</v>
       </c>
-      <c r="P2" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="R2" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>16</v>
       </c>
@@ -758,67 +792,67 @@
         <v>0</v>
       </c>
       <c r="C3" t="s">
+        <v>47</v>
+      </c>
+      <c r="D3" t="s">
         <v>50</v>
-      </c>
-      <c r="D3" t="s">
-        <v>53</v>
       </c>
       <c r="E3" t="s">
         <v>25</v>
       </c>
-      <c r="O3" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>16</v>
       </c>
       <c r="B4" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C4" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="D4" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="E4" t="s">
         <v>26</v>
       </c>
-      <c r="O4" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="Q4" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>16</v>
       </c>
       <c r="B5" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C5" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="E5" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="6" spans="1:16" ht="34" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:18" ht="34" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>17</v>
       </c>
       <c r="B6" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="E6" t="s">
         <v>24</v>
@@ -827,32 +861,41 @@
         <v>20</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="K6" s="1"/>
       <c r="L6" s="1"/>
-      <c r="M6" t="s">
-        <v>42</v>
-      </c>
-      <c r="P6" s="2" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="7" spans="1:16" ht="34" x14ac:dyDescent="0.2">
+      <c r="M6" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="N6" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="O6" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>43</v>
+      </c>
+      <c r="R6" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>17</v>
       </c>
       <c r="B7" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="E7" t="s">
         <v>23</v>
@@ -864,27 +907,28 @@
         <v>22</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="M7" t="s">
+        <v>54</v>
+      </c>
+      <c r="M7" t="b">
+        <v>1</v>
+      </c>
+      <c r="O7" t="s">
         <v>59</v>
       </c>
-      <c r="N7">
+      <c r="P7">
         <v>1</v>
       </c>
-      <c r="P7" s="2" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="R7" s="1"/>
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>18</v>
       </c>
       <c r="B8" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>2</v>
@@ -899,31 +943,34 @@
         <v>30</v>
       </c>
       <c r="I8" s="1"/>
-      <c r="M8" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="O8" t="s">
+        <v>56</v>
+      </c>
+      <c r="Q8" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>18</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="D9" s="1"/>
       <c r="G9" s="1"/>
       <c r="H9" s="1"/>
       <c r="I9" s="1"/>
     </row>
-    <row r="10" spans="1:16" ht="34" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:18" ht="34" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>18</v>
       </c>
       <c r="B10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>3</v>
@@ -932,13 +979,13 @@
         <v>31</v>
       </c>
       <c r="F10" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>32</v>
+        <v>63</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>33</v>
+        <v>62</v>
       </c>
       <c r="I10" s="1"/>
       <c r="J10" s="1" t="s">
@@ -950,19 +997,28 @@
       <c r="L10" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="P10" s="3" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="11" spans="1:16" ht="34" x14ac:dyDescent="0.2">
+      <c r="M10" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="N10" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q10" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="R10" s="3" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>18</v>
       </c>
       <c r="B11" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="D11" s="1" t="s">
         <v>3</v>
@@ -971,43 +1027,46 @@
         <v>31</v>
       </c>
       <c r="F11" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>32</v>
+        <v>63</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="I11" s="1"/>
+        <v>62</v>
+      </c>
+      <c r="I11" s="1" t="s">
+        <v>64</v>
+      </c>
       <c r="J11" s="1" t="s">
-        <v>4</v>
+        <v>67</v>
       </c>
       <c r="K11" s="1" t="s">
-        <v>5</v>
+        <v>66</v>
       </c>
       <c r="L11" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="P11" s="3" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="M11" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="N11" s="1"/>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>18</v>
       </c>
       <c r="B12" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="E12" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="G12" s="1"/>
       <c r="H12" s="1"/>
@@ -1015,6 +1074,48 @@
       <c r="J12" s="1"/>
       <c r="K12" s="1"/>
       <c r="L12" s="1"/>
+      <c r="M12" s="1"/>
+      <c r="N12" s="1"/>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>18</v>
+      </c>
+      <c r="B13" t="s">
+        <v>72</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E13" t="s">
+        <v>31</v>
+      </c>
+      <c r="F13" t="s">
+        <v>39</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="H13" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="I13" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="J13" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="K13" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="L13" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="M13" s="1"/>
+      <c r="N13" s="1"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>

</xml_diff>